<commit_message>
Changes to address reviewers comments
</commit_message>
<xml_diff>
--- a/results/tab/trait_trait_mixed_models_sheets_global.xlsx
+++ b/results/tab/trait_trait_mixed_models_sheets_global.xlsx
@@ -1,30 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rbgkew-my.sharepoint.com/personal/j_white2_kew_org/Documents/Documents/research/colabs/drakensberg_grasslands_functional_traits/results/tab/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://miamiedu-my.sharepoint.com/personal/lxa1960_miami_edu/Documents/UMiami/PFTC7/drakensberg_grasslands_functional_traits/results/tab/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="106" documentId="11_8925DCD38F79A8D366075C52F37BD272AAC71092" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B99DD0C-75F0-4CC4-893C-21153F1F2A14}"/>
+  <xr:revisionPtr revIDLastSave="145" documentId="11_8925DCD38F79A8D366075C52F37BD272AAC71092" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9120CDE9-93FA-436D-BB8F-305CB4A0CB2D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Analogous traits" sheetId="1" r:id="rId1"/>
     <sheet name="Leaf-leaf and root-root traits" sheetId="5" r:id="rId2"/>
     <sheet name="PFTC7 Leaf-leaf traits" sheetId="3" r:id="rId3"/>
     <sheet name="Plant size traits" sheetId="2" r:id="rId4"/>
-    <sheet name="Additional information" sheetId="4" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId5"/>
+    <sheet name="Additional information" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="252">
   <si>
     <t>A. leaf thickness~sla (linear)</t>
   </si>
@@ -729,6 +730,57 @@
   </si>
   <si>
     <t>C. ldmc~rtd (polynomial)</t>
+  </si>
+  <si>
+    <t>D. leaf thickness~sla (linear)</t>
+  </si>
+  <si>
+    <t>E. ldmc~sla (polynomial)</t>
+  </si>
+  <si>
+    <t>F. ldmc~leaf thickness (polynomial)</t>
+  </si>
+  <si>
+    <t>G. rd~srl (linear)</t>
+  </si>
+  <si>
+    <t>H. rtd~srl (polynomial)</t>
+  </si>
+  <si>
+    <t>I. rtd~rd (linear)</t>
+  </si>
+  <si>
+    <t>J. leaf thickness~sla (linear)</t>
+  </si>
+  <si>
+    <t>K. ldmc~sla (polynomial)</t>
+  </si>
+  <si>
+    <t>L. ldmc~leaf thickness (linear)</t>
+  </si>
+  <si>
+    <t>M. aboveground biomass~belowground biomass (linear)</t>
+  </si>
+  <si>
+    <t>N. veg height~root depth (linear)</t>
+  </si>
+  <si>
+    <t>O. root depth~belowground biomass (linear)</t>
+  </si>
+  <si>
+    <t>P. srl~belowground biomass (linear)</t>
+  </si>
+  <si>
+    <t>Q. sla~belowground biomass (polynomial)</t>
+  </si>
+  <si>
+    <t>R. veg height~aboveground biomass (polynomial)</t>
+  </si>
+  <si>
+    <t>S. srl~aboveground biomass (linear)</t>
+  </si>
+  <si>
+    <t>T. sla~aboveground biomass (polynomial)</t>
   </si>
 </sst>
 </file>
@@ -792,10 +844,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1086,20 +1134,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="30.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="30.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>221</v>
       </c>
@@ -1146,7 +1194,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>232</v>
       </c>
@@ -1187,7 +1235,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>233</v>
       </c>
@@ -1228,7 +1276,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>234</v>
       </c>
@@ -1283,15 +1331,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{648453A0-9DC0-4CCC-A319-113634939275}">
   <dimension ref="A1:O7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>221</v>
       </c>
@@ -1338,7 +1386,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1376,7 +1424,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1423,7 +1471,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1464,7 +1512,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1502,7 +1550,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1549,7 +1597,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1592,18 +1640,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{140FCD34-926D-49EC-AC57-EA5202DA1F89}">
   <dimension ref="A1:O4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="28.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="28.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="28.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>221</v>
       </c>
@@ -1650,7 +1698,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1694,7 +1742,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1741,7 +1789,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>219</v>
       </c>
@@ -1793,21 +1841,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A58C3EE-38DA-4749-B02E-E8C9127C4435}">
   <dimension ref="A1:M9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="51.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="51.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="41.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="33.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="38.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="45.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="33.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="51.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="51.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="41.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="38.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="45.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="33.88671875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="39" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>221</v>
       </c>
@@ -1848,7 +1896,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>116</v>
       </c>
@@ -1886,7 +1934,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>117</v>
       </c>
@@ -1924,7 +1972,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>118</v>
       </c>
@@ -1962,7 +2010,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>119</v>
       </c>
@@ -2000,7 +2048,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>120</v>
       </c>
@@ -2041,7 +2089,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>121</v>
       </c>
@@ -2082,7 +2130,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>122</v>
       </c>
@@ -2117,7 +2165,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>123</v>
       </c>
@@ -2164,56 +2212,948 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01EC6EDF-D7E9-4928-9C9A-A4BDE82DCC7C}">
+  <dimension ref="A1:O21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="47.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="3.77734375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>232</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I2" t="s">
+        <v>69</v>
+      </c>
+      <c r="J2" t="s">
+        <v>77</v>
+      </c>
+      <c r="L2" t="s">
+        <v>90</v>
+      </c>
+      <c r="M2" t="s">
+        <v>100</v>
+      </c>
+      <c r="O2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>233</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H3" t="s">
+        <v>66</v>
+      </c>
+      <c r="I3" t="s">
+        <v>69</v>
+      </c>
+      <c r="J3" t="s">
+        <v>78</v>
+      </c>
+      <c r="L3" t="s">
+        <v>91</v>
+      </c>
+      <c r="M3" t="s">
+        <v>101</v>
+      </c>
+      <c r="O3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>234</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" t="s">
+        <v>41</v>
+      </c>
+      <c r="F4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G4" t="s">
+        <v>57</v>
+      </c>
+      <c r="H4" t="s">
+        <v>67</v>
+      </c>
+      <c r="I4" t="s">
+        <v>69</v>
+      </c>
+      <c r="J4" t="s">
+        <v>79</v>
+      </c>
+      <c r="K4" t="s">
+        <v>82</v>
+      </c>
+      <c r="L4" t="s">
+        <v>92</v>
+      </c>
+      <c r="M4" t="s">
+        <v>102</v>
+      </c>
+      <c r="N4" t="s">
+        <v>106</v>
+      </c>
+      <c r="O4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>235</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G5" t="s">
+        <v>53</v>
+      </c>
+      <c r="H5" t="s">
+        <v>59</v>
+      </c>
+      <c r="I5" t="s">
+        <v>69</v>
+      </c>
+      <c r="J5" t="s">
+        <v>71</v>
+      </c>
+      <c r="L5" t="s">
+        <v>84</v>
+      </c>
+      <c r="M5" t="s">
+        <v>94</v>
+      </c>
+      <c r="O5" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>236</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" t="s">
+        <v>44</v>
+      </c>
+      <c r="G6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H6" t="s">
+        <v>60</v>
+      </c>
+      <c r="I6" t="s">
+        <v>69</v>
+      </c>
+      <c r="J6" t="s">
+        <v>72</v>
+      </c>
+      <c r="K6" t="s">
+        <v>81</v>
+      </c>
+      <c r="L6" t="s">
+        <v>85</v>
+      </c>
+      <c r="M6" t="s">
+        <v>95</v>
+      </c>
+      <c r="N6" t="s">
+        <v>104</v>
+      </c>
+      <c r="O6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>237</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G7" t="s">
+        <v>53</v>
+      </c>
+      <c r="H7" t="s">
+        <v>61</v>
+      </c>
+      <c r="I7" t="s">
+        <v>69</v>
+      </c>
+      <c r="J7" t="s">
+        <v>73</v>
+      </c>
+      <c r="L7" t="s">
+        <v>86</v>
+      </c>
+      <c r="M7" t="s">
+        <v>96</v>
+      </c>
+      <c r="O7" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>238</v>
+      </c>
+      <c r="B8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" t="s">
+        <v>46</v>
+      </c>
+      <c r="G8" t="s">
+        <v>53</v>
+      </c>
+      <c r="H8" t="s">
+        <v>62</v>
+      </c>
+      <c r="I8" t="s">
+        <v>69</v>
+      </c>
+      <c r="J8" t="s">
+        <v>74</v>
+      </c>
+      <c r="L8" t="s">
+        <v>87</v>
+      </c>
+      <c r="M8" t="s">
+        <v>97</v>
+      </c>
+      <c r="O8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>239</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9" t="s">
+        <v>55</v>
+      </c>
+      <c r="H9" t="s">
+        <v>63</v>
+      </c>
+      <c r="I9" t="s">
+        <v>69</v>
+      </c>
+      <c r="J9" t="s">
+        <v>75</v>
+      </c>
+      <c r="K9" t="s">
+        <v>71</v>
+      </c>
+      <c r="L9" t="s">
+        <v>88</v>
+      </c>
+      <c r="M9" t="s">
+        <v>98</v>
+      </c>
+      <c r="N9" t="s">
+        <v>105</v>
+      </c>
+      <c r="O9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>240</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F10" t="s">
+        <v>48</v>
+      </c>
+      <c r="H10" t="s">
+        <v>64</v>
+      </c>
+      <c r="I10" t="s">
+        <v>69</v>
+      </c>
+      <c r="J10" t="s">
+        <v>76</v>
+      </c>
+      <c r="L10" t="s">
+        <v>89</v>
+      </c>
+      <c r="M10" t="s">
+        <v>99</v>
+      </c>
+      <c r="O10" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>241</v>
+      </c>
+      <c r="B11" t="s">
+        <v>218</v>
+      </c>
+      <c r="C11" t="s">
+        <v>215</v>
+      </c>
+      <c r="E11" t="s">
+        <v>211</v>
+      </c>
+      <c r="F11" t="s">
+        <v>209</v>
+      </c>
+      <c r="G11" t="s">
+        <v>206</v>
+      </c>
+      <c r="H11" t="s">
+        <v>78</v>
+      </c>
+      <c r="I11" t="s">
+        <v>201</v>
+      </c>
+      <c r="J11" t="s">
+        <v>200</v>
+      </c>
+      <c r="K11" t="s">
+        <v>198</v>
+      </c>
+      <c r="L11" t="s">
+        <v>195</v>
+      </c>
+      <c r="M11" t="s">
+        <v>192</v>
+      </c>
+      <c r="N11" t="s">
+        <v>189</v>
+      </c>
+      <c r="O11" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>242</v>
+      </c>
+      <c r="B12" t="s">
+        <v>217</v>
+      </c>
+      <c r="C12" t="s">
+        <v>214</v>
+      </c>
+      <c r="D12" t="s">
+        <v>212</v>
+      </c>
+      <c r="E12" t="s">
+        <v>210</v>
+      </c>
+      <c r="F12" t="s">
+        <v>208</v>
+      </c>
+      <c r="G12" t="s">
+        <v>205</v>
+      </c>
+      <c r="H12" t="s">
+        <v>203</v>
+      </c>
+      <c r="I12" t="s">
+        <v>201</v>
+      </c>
+      <c r="J12" t="s">
+        <v>169</v>
+      </c>
+      <c r="K12" t="s">
+        <v>197</v>
+      </c>
+      <c r="L12" t="s">
+        <v>194</v>
+      </c>
+      <c r="M12" t="s">
+        <v>191</v>
+      </c>
+      <c r="N12" t="s">
+        <v>104</v>
+      </c>
+      <c r="O12" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>243</v>
+      </c>
+      <c r="B13" t="s">
+        <v>216</v>
+      </c>
+      <c r="C13" t="s">
+        <v>213</v>
+      </c>
+      <c r="E13" t="s">
+        <v>158</v>
+      </c>
+      <c r="F13" t="s">
+        <v>207</v>
+      </c>
+      <c r="G13" t="s">
+        <v>204</v>
+      </c>
+      <c r="H13" t="s">
+        <v>202</v>
+      </c>
+      <c r="I13" t="s">
+        <v>201</v>
+      </c>
+      <c r="J13" t="s">
+        <v>199</v>
+      </c>
+      <c r="K13" t="s">
+        <v>196</v>
+      </c>
+      <c r="L13" t="s">
+        <v>193</v>
+      </c>
+      <c r="M13" t="s">
+        <v>190</v>
+      </c>
+      <c r="N13" t="s">
+        <v>106</v>
+      </c>
+      <c r="O13" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>244</v>
+      </c>
+      <c r="B14" t="s">
+        <v>124</v>
+      </c>
+      <c r="C14" t="s">
+        <v>132</v>
+      </c>
+      <c r="E14" t="s">
+        <v>143</v>
+      </c>
+      <c r="F14" t="s">
+        <v>149</v>
+      </c>
+      <c r="G14" t="s">
+        <v>56</v>
+      </c>
+      <c r="H14" t="s">
+        <v>156</v>
+      </c>
+      <c r="I14" t="s">
+        <v>162</v>
+      </c>
+      <c r="J14" t="s">
+        <v>163</v>
+      </c>
+      <c r="K14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L14" t="s">
+        <v>178</v>
+      </c>
+      <c r="M14" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>245</v>
+      </c>
+      <c r="B15" t="s">
+        <v>125</v>
+      </c>
+      <c r="C15" t="s">
+        <v>133</v>
+      </c>
+      <c r="E15" t="s">
+        <v>144</v>
+      </c>
+      <c r="F15" t="s">
+        <v>150</v>
+      </c>
+      <c r="G15" t="s">
+        <v>53</v>
+      </c>
+      <c r="H15" t="s">
+        <v>157</v>
+      </c>
+      <c r="I15" t="s">
+        <v>162</v>
+      </c>
+      <c r="J15" t="s">
+        <v>164</v>
+      </c>
+      <c r="K15" t="s">
+        <v>171</v>
+      </c>
+      <c r="L15" t="s">
+        <v>179</v>
+      </c>
+      <c r="M15" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>246</v>
+      </c>
+      <c r="B16" t="s">
+        <v>126</v>
+      </c>
+      <c r="C16" t="s">
+        <v>134</v>
+      </c>
+      <c r="E16" t="s">
+        <v>145</v>
+      </c>
+      <c r="F16" t="s">
+        <v>151</v>
+      </c>
+      <c r="G16" t="s">
+        <v>56</v>
+      </c>
+      <c r="H16" t="s">
+        <v>158</v>
+      </c>
+      <c r="I16" t="s">
+        <v>162</v>
+      </c>
+      <c r="J16" t="s">
+        <v>41</v>
+      </c>
+      <c r="K16" t="s">
+        <v>172</v>
+      </c>
+      <c r="L16" t="s">
+        <v>180</v>
+      </c>
+      <c r="M16" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>247</v>
+      </c>
+      <c r="B17" t="s">
+        <v>127</v>
+      </c>
+      <c r="C17" t="s">
+        <v>135</v>
+      </c>
+      <c r="E17" t="s">
+        <v>38</v>
+      </c>
+      <c r="F17" t="s">
+        <v>38</v>
+      </c>
+      <c r="G17" t="s">
+        <v>155</v>
+      </c>
+      <c r="H17" t="s">
+        <v>159</v>
+      </c>
+      <c r="I17" t="s">
+        <v>162</v>
+      </c>
+      <c r="J17" t="s">
+        <v>165</v>
+      </c>
+      <c r="K17" t="s">
+        <v>173</v>
+      </c>
+      <c r="L17" t="s">
+        <v>181</v>
+      </c>
+      <c r="M17" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>248</v>
+      </c>
+      <c r="B18" t="s">
+        <v>128</v>
+      </c>
+      <c r="C18" t="s">
+        <v>136</v>
+      </c>
+      <c r="D18" t="s">
+        <v>140</v>
+      </c>
+      <c r="E18" t="s">
+        <v>146</v>
+      </c>
+      <c r="F18" t="s">
+        <v>152</v>
+      </c>
+      <c r="G18" t="s">
+        <v>53</v>
+      </c>
+      <c r="H18" t="s">
+        <v>160</v>
+      </c>
+      <c r="I18" t="s">
+        <v>162</v>
+      </c>
+      <c r="J18" t="s">
+        <v>166</v>
+      </c>
+      <c r="K18" t="s">
+        <v>174</v>
+      </c>
+      <c r="L18" t="s">
+        <v>182</v>
+      </c>
+      <c r="M18" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>249</v>
+      </c>
+      <c r="B19" t="s">
+        <v>129</v>
+      </c>
+      <c r="C19" t="s">
+        <v>137</v>
+      </c>
+      <c r="D19" t="s">
+        <v>141</v>
+      </c>
+      <c r="E19" t="s">
+        <v>147</v>
+      </c>
+      <c r="F19" t="s">
+        <v>153</v>
+      </c>
+      <c r="G19" t="s">
+        <v>53</v>
+      </c>
+      <c r="H19" t="s">
+        <v>161</v>
+      </c>
+      <c r="I19" t="s">
+        <v>162</v>
+      </c>
+      <c r="J19" t="s">
+        <v>167</v>
+      </c>
+      <c r="K19" t="s">
+        <v>175</v>
+      </c>
+      <c r="L19" t="s">
+        <v>183</v>
+      </c>
+      <c r="M19" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>250</v>
+      </c>
+      <c r="B20" t="s">
+        <v>130</v>
+      </c>
+      <c r="C20" t="s">
+        <v>138</v>
+      </c>
+      <c r="E20" t="s">
+        <v>38</v>
+      </c>
+      <c r="F20" t="s">
+        <v>38</v>
+      </c>
+      <c r="H20" t="s">
+        <v>46</v>
+      </c>
+      <c r="I20" t="s">
+        <v>162</v>
+      </c>
+      <c r="J20" t="s">
+        <v>168</v>
+      </c>
+      <c r="K20" t="s">
+        <v>176</v>
+      </c>
+      <c r="L20" t="s">
+        <v>184</v>
+      </c>
+      <c r="M20" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>251</v>
+      </c>
+      <c r="B21" t="s">
+        <v>131</v>
+      </c>
+      <c r="C21" t="s">
+        <v>139</v>
+      </c>
+      <c r="D21" t="s">
+        <v>142</v>
+      </c>
+      <c r="E21" t="s">
+        <v>148</v>
+      </c>
+      <c r="F21" t="s">
+        <v>154</v>
+      </c>
+      <c r="G21" t="s">
+        <v>53</v>
+      </c>
+      <c r="H21" t="s">
+        <v>160</v>
+      </c>
+      <c r="I21" t="s">
+        <v>162</v>
+      </c>
+      <c r="J21" t="s">
+        <v>169</v>
+      </c>
+      <c r="K21" t="s">
+        <v>177</v>
+      </c>
+      <c r="L21" t="s">
+        <v>185</v>
+      </c>
+      <c r="M21" t="s">
+        <v>112</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A048CF41-BDF9-405C-A7A9-49C70F86973E}">
   <dimension ref="A1:A10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>230</v>
       </c>

</xml_diff>